<commit_message>
Leads: 2026-10-02 00:03 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Air Conditioning Installation Torrance, CA | Same Day Service</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>acfixca.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://acfixca.com/torrance-ca/air-conditioning-installation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Serving All</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>info@acfixca.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(858) 392-8090</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>AC installation Torrance CA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:05 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cabrillo Plumbing, Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>discovercabrillo.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://discovercabrillo.com/heat-pump/heat-pump-installation-replacement-san-francisco-ca</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Water Heaters</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>support@discovercabrillo.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(415) 843-2900</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>heat pump installation San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:06 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>702 Roofing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>702roofing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.702roofing.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Founder John</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@702roofing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>702-551-5715</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>86</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofing contractor Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:12 UTC (cycle 136)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>316 EXTERIORS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>316exteriors.us</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://316exteriors.us/location/springfield/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Cole County</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>316extoffice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(573) 826-7843</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Springfield MO</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofing contractor Springfield MO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:21 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Landmark Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>landmarkroof.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://landmarkroof.com/everett-roofing-and-siding-contractor</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Flexible Financing</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@landmarkroof.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>855-908-7663</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Everett WA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>residential roofing company Everett WA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:24 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -863,6 +863,62 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HVAC Services | Comforts on the Coast</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>comfortsonthecoast.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.comfortsonthecoast.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>andrea.mannon@cotc-llc.net</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(228) 236-4822</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Biloxi MS</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>air conditioning repair Biloxi MS</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:25 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -884,7 +884,6 @@
           <t>https://www.comfortsonthecoast.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>andrea.mannon@cotc-llc.net</t>
@@ -914,6 +913,62 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>APC Service Pros</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>apcservicepros.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://apcservicepros.com/san-marcos-ac-repair</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@apcservicepros.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>512-410-7739</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>air conditioning repair San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:30 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -939,7 +939,6 @@
           <t>https://apcservicepros.com/san-marcos-ac-repair</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>info@apcservicepros.com</t>
@@ -969,6 +968,126 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>causewayplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.causewayplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Hampton Roads</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>dave@causewayplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>757-582-9259</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>plumbing company Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3D Exteriors: Expert Roofing &amp; Exterior Solutions in Portland, ME</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3dexteriors.me</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://3dexteriors.me/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Lakes Region</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>jdyer@3dexteriors.me</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(207)-739-9228</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Portland ME</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roof replacement Portland ME</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:31 UTC (cycle 149)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1093,6 +1093,122 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tulsa Roofing &amp; Roof Repair</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>tulsaroofco.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://tulsaroofco.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@tulsaroofco.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>918-205-9661</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roof repair company Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>4L Contracting LLC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>4lcontractingllc.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://4lcontractingllc.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Team Led</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>service@4lcontractingllc.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>979-473-9775</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>water heater repair College Station TX</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:34 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1114,7 +1114,6 @@
           <t>https://tulsaroofco.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>info@tulsaroofco.com</t>
@@ -1204,6 +1203,62 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Blue Planet Plumbing</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>plumbersinsandiego.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://plumbersinsandiego.com/sewer-line-repair-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@blueplanetsd.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>858) 914-4696</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>sewer repair San Diego CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:36 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1229,7 +1229,6 @@
           <t>https://plumbersinsandiego.com/sewer-line-repair-and-replacement/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>info@blueplanetsd.com</t>
@@ -1259,6 +1258,122 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Dakota Roofing</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>dakotaroofingnw.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://dakotaroofingnw.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Trusted Roofin</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@dakotaroofingnw.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>503-394-2615</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roof replacement Salem OR</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Air Supply</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>airsupplyhammond.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.airsupplyhammond.com/services</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>airsupply1978@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(985) 402-3365</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Hammond IN</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>76</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>heat pump installation Hammond IN</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:42 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1344,7 +1344,6 @@
           <t>https://www.airsupplyhammond.com/services</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>airsupply1978@gmail.com</t>
@@ -1374,6 +1373,63 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>All Systems Heating 
+and Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>allsystemsheatac.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://allsystemsheatac.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@indiantypefoundry.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>732-908-0428</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>HVAC contractor Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:50 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1400,7 +1400,6 @@
           <t>https://allsystemsheatac.com/</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>info@indiantypefoundry.com</t>
@@ -1430,6 +1429,122 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Douglas Orr Plumbing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>orrplumbing.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://orrplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Plumbing Problems</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@orrplumbing.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>305-240-6731</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>plumbing company Miami FL</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AAA Pro Plumbing</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>aaaproplumbing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://aaaproplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@aaaproplumbing.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(786) 273-0577</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>plumbing company Miami FL</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:55 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1515,7 +1515,6 @@
           <t>https://aaaproplumbing.com/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>info@aaaproplumbing.com</t>
@@ -1545,6 +1544,66 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Green Factor</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>gfipro.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.gfipro.com/home-services/hvac/heat-pump/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Factor For</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@gfipro.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>785.256.9443</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Lawrence KS</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>heat pump installation Lawrence KS</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 00:59 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1609,6 +1609,62 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Optimal Heating and Air</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>optimalheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://optimalheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@optimalheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(661) 319-4258</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>air conditioning repair Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:05 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1630,7 +1630,6 @@
           <t>https://optimalheatingandair.com/</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>info@optimalheatingandair.com</t>
@@ -1660,6 +1659,126 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Killeen, TX</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>atxroofings.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://atxroofings.com/killeen-tx/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>atxroofinghomesolutions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(512)269-2397</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Killeen TX</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>residential roofing company Killeen TX</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HVAC Repair and Replacement</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>truepros.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://truepros.com/west-valley-city/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Why West</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info@truepros.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(385) 209-1730</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>West Valley City UT</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>furnace repair West Valley City UT</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:14 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1784,6 +1784,186 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ArcCon Roofing and Construction Services</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>arcconroofing.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.arcconroofing.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Tornado Victim</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>charlie@arcconbuilding.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(205) 335-8344</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>roofing contractor Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Higher Roof Solutions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>higherroofsolutions.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://higherroofsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Higher Roof</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>john@higherroofsolutions.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(205) 386-0565</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>roofing contractor Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Abide Roofing | Birmingham, AL Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>abideroof.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.abideroof.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Emergency Repair</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>info@abideroof.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>205.577.7338</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>76</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>roofing contractor Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:28 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1964,6 +1964,66 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ideal Air Conditioning &amp; Insulation</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>idealairaz.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://idealairaz.com/air-conditioning/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Pumps Top</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>info@idealairaz.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(480) 839-0082</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>heat pump installation Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:33 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2024,6 +2024,62 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Drain Cleaning | Clog &amp; Obstruction Removal | Hilo, HI</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>hilopumpingservice.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>http://www.hilopumpingservice.com/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>hilopumpingservice@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>808-938-0454</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Hilo HI</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>68</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>drain cleaning service Hilo HI</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:36 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2045,7 +2045,6 @@
           <t>http://www.hilopumpingservice.com/drain-cleaning</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>hilopumpingservice@yahoo.com</t>
@@ -2075,6 +2074,118 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Queens &amp; Brooklyn, NYC Sewer &amp; Drain Plumbers</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>plumberinqueens.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.plumberinqueens.com/plumbing-sewer-drain-cleaning-nyc/queens-sewer-drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>info@plumberinqueens.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>718-729-4995</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>drain cleaning service Queens NY</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Metal Roofing | Asheville, NC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>jeffsroofingasheville.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.jeffsroofingasheville.com/metal-roofers</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>jeffsroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(828) 779-3472</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Asheville NC</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:37 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2100,7 +2100,6 @@
           <t>https://www.plumberinqueens.com/plumbing-sewer-drain-cleaning-nyc/queens-sewer-drain-cleaning/</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>info@plumberinqueens.com</t>
@@ -2156,7 +2155,6 @@
           <t>https://www.jeffsroofingasheville.com/metal-roofers</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>jeffsroofinginc@gmail.com</t>
@@ -2186,6 +2184,66 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>nuflowalaska</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>nuflowalaska.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.nuflowalaska.com/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Nu Flow</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>info@nuflowalaska.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(907) 677-2145</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>drain cleaning service Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:39 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2249,6 +2249,126 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Masonboro Air</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>masonboroair.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.masonboroair.com/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Masonboro Air</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>office@masonboroair.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(910) 530-2033</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>HVAC contractor Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Raptorroofs</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>raptorroofs.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.raptorroofs.com/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Jaykob Hi</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>info@raptorroofs.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(502) 576-4343</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>88</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Louisville KY</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:40 UTC (cycle 196)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2369,6 +2369,62 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Budget Sewer Service -</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>budgetsewerservice.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://budgetsewerservice.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>dispatcher@budgetsewerservice.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>706-798-8080</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Augusta GA</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>82</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>drain cleaning service Augusta GA</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:45 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2390,7 +2390,6 @@
           <t>https://budgetsewerservice.com/</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>dispatcher@budgetsewerservice.com</t>
@@ -2420,6 +2419,62 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Andrews Heating &amp; Cooling, LLC</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>andrewsheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.andrewsheatingcooling.com/boiler-and-furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>info@andrewsheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>262-456-6156</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Racine WI</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>furnace repair Racine WI</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 01:48 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2445,7 +2445,6 @@
           <t>https://www.andrewsheatingcooling.com/boiler-and-furnace-repair/</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>info@andrewsheatingcooling.com</t>
@@ -2475,6 +2474,62 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>C &amp; C Service | HVAC Contractor | Heating &amp; Air Conditioning Repair &amp; Service</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ccservicellc.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.ccservicellc.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>service@hpcmechanical.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>203-323-2866</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>96</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>heating and cooling company Stamford CT</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 14:38 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2500,7 +2500,6 @@
           <t>https://www.ccservicellc.com/</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>service@hpcmechanical.com</t>
@@ -2530,6 +2529,126 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Roofing Services | Murphy &amp; Sons Roofing | Kansas City</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>murphyroofing.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://murphyroofing.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Leavenworth County</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>murphyroofing@kc.rr.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(913) 287-2116</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>roof replacement Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Alexanders Roofing</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>alexanders-roofing.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.alexanders-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sam Alexander</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>info@alexanders-roofing.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(816) 698-9115</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>90</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roof replacement Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 14:41 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2654,6 +2654,66 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Richardson Plumbing Company</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>richardsonplumbing.net</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.richardsonplumbing.net/hot-water-system-supplier/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Home About</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>richardsonplmb@gmail.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(515) 306-1205</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Des Moines IA</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>water heater repair Des Moines IA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 14:42 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2714,6 +2714,62 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sewer repair</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>plumbercarrolltontx.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://plumbercarrolltontx.com/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>service@plumbercarrolltontx.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>972-591-3869</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>sewer repair Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 14:44 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2735,7 +2735,6 @@
           <t>https://plumbercarrolltontx.com/sewer-repair/</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>service@plumbercarrolltontx.com</t>
@@ -2765,6 +2764,122 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HVAC Surprise, AZ | AC &amp; Heating Repair | B &amp; E Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>beheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://beheatingcooling.com/service-area/surprise-az/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>info@beheatingandcooling.net</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(602) 281-6610</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Surprise AZ</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>100</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>heating and cooling company Surprise AZ</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Drew's Plumbing Inc.</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>drewsplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.drewsplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Ryan Selner</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>contact@drewsplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>920-371-6098</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Green Bay WI</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>plumbing company Green Bay WI</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 14:45 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2790,7 +2790,6 @@
           <t>https://beheatingcooling.com/service-area/surprise-az/</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>info@beheatingandcooling.net</t>
@@ -2880,6 +2879,126 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Talmich Plumbing and Heating</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>talmichplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://talmichplumbingheating.com/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Colorado Springs</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>contact@talmichplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(719) 822-0448</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>plumber Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AC Pros</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>acprosnmb.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://acprosnmb.com/services/hvac-installations-myrtle-beach-south-carolina/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Who We</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>chris@acprosnmb.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(843) 445-2592</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>100</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>AC installation Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 14:50 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3004,6 +3004,122 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>California Bay Roofing Inc</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>californiabayroofinginc.net</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.californiabayroofinginc.net/fremont-roofing</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>amcalroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(415) 684-4498</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>roof replacement Fremont CA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>AC Repair &amp; HVAC in Pembroke Pines, FL | Power Air</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>powerairac.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://powerairac.com/areas/pembroke-pines</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>info@powerairac.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(305) 761-0023</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>100</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>air conditioning repair Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:02 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3025,7 +3025,6 @@
           <t>https://www.californiabayroofinginc.net/fremont-roofing</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>amcalroofinginc@gmail.com</t>
@@ -3115,6 +3114,66 @@
         </is>
       </c>
       <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>HVAC Alliance Expert</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>hvacallianceexpert.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://hvacallianceexpert.com/locations/pembroke-pines/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Helping Home</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@hvacallianceexpert.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(754) 253-3535</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>100</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HVAC contractor Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:03 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3179,6 +3179,66 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Elite Services &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>eliteservicesandroofing.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://eliteservicesandroofing.com/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Featured Post</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>derek.esroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>385-600-7672</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>100</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Ogden UT</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:11 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3239,6 +3239,66 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Fresno &amp; Clovis Plumbers | Art Douglas Plumbing | Since 1971</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>artdouglasplumbing.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.artdouglasplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>dispatch@artdouglasplumbing.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>559-291-7230</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>plumber Fresno CA</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:12 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3299,6 +3299,66 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Plumber | Des Moines, IA | H &amp; H Plumbing Inc</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>handhplumbing.net</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.handhplumbing.net/plumber-des-moines-ia</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Moines Neighborhoods</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>handhplumbinginc@aol.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(515) 277-5755</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Des Moines IA</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>90</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>plumber Des Moines IA</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:15 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3359,6 +3359,242 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Rooftops Energy Solutions</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>rooftopses.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://rooftopses.com/service-area/treasure-valley/roofer-meridian/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Treasure Valley</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>operations@rooftopses.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(208) 870-1584</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Meridian ID</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>100</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>roofer Meridian ID</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Wimpy's Plumbing &amp; Air</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>wimpysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.wimpysplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>info@lovewimpys.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(941) 294-3214</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>98</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>plumbing company Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>home - Sarasota, FL - Barriere Plumbing</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>barriereplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.barriereplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>barrieretbp2@aol.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>941-423-8223</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>plumbing company Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Boise Roofing Company</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>sawtooth-roofing.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://sawtooth-roofing.com/boise-roofing</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Treasure Val</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>contact@sawtooth-roofing.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>208.996.8748</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>roof repair company Boise ID</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:24 UTC (cycle 33)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3500,7 +3500,6 @@
           <t>https://www.barriereplumbinginc.com/</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>barrieretbp2@aol.com</t>
@@ -3590,6 +3589,66 @@
         </is>
       </c>
       <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>QNK Roofing</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>qnkroofing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.qnkroofing.com/stamford-ct/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Stamford Greenwich</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>info@qnkroofing.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(203) 883-5033</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>100</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>residential roofing company Stamford CT</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:34 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3654,6 +3654,66 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Water Heater Repair in Annapolis, MD | Carter Quality Plumbing</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>carterqualityplumbing.net</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.carterqualityplumbing.net/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Anne Arundel</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>brian@carterqualityplumbing.net</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(410) 705-2589</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>water heater repair Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:39 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3714,6 +3714,66 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Pickle Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>pickleroofing.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://pickleroofing.com/roof-replacement-contractor-richardson-tx</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>What Homeowners</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>info@pickleroofing.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(972) 954-7186</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>100</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>roof replacement Richardson TX</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:40 UTC (cycle 44)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3774,6 +3774,66 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Pro-Tech HVAC Home</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>protechhvachome.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://protechhvachome.com/heat-pump-installation-replacement-annapolis/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>How Does</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>office@protechhvachome.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(240) 298-6521</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>100</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>heat pump installation Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:45 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3834,6 +3834,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Residential Roofing Installation &amp; Repair | Hartford, CT</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>allhomeimprovementsct.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.allhomeimprovementsct.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Request Estimate</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>allhomeimprovements26@gmail.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(860) 222-2546</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Hartford CT</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>88</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>residential roofing company Hartford CT</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:46 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3894,6 +3894,62 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Bill's Plumbing and Heating LLC Contact us at (218) 590-2104 - Contact us at (21</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>billsplumbingmn.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://billsplumbingmn.com/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>tony@billsplumbingmn.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(218) 590-2104</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>90</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>plumber Duluth MN</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:48 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3915,7 +3915,6 @@
           <t>https://billsplumbingmn.com/</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>tony@billsplumbingmn.com</t>
@@ -3945,6 +3944,62 @@
         </is>
       </c>
       <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Expert Furnace &amp; HVAC Services in Bellingham | AirTech HVAC</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>airtechheat.net</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.airtechheat.net/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>hydromechanical@msn.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>360-734-5010</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>88</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>heat pump installation Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:51 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3970,7 +3970,6 @@
           <t>https://www.airtechheat.net/</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>hydromechanical@msn.com</t>
@@ -4000,6 +3999,62 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Olathe</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>searingelectricandplumbing.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.searingelectricandplumbing.com/locations/olathe-ks/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>info@searingelectricandplumbing.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(833) 336-1231</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>drain cleaning service Olathe KS</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 15:52 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4025,7 +4025,6 @@
           <t>https://www.searingelectricandplumbing.com/locations/olathe-ks/drain-cleaning</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>info@searingelectricandplumbing.com</t>
@@ -4055,6 +4054,66 @@
         </is>
       </c>
       <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>HVAC Newark DE</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>hvacnewarkde.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://hvacnewarkde.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Locally Owned</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>service@hvacnewarkde.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(327) 210-5999</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Newark DE</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>100</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>HVAC contractor Newark DE</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:05 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4119,6 +4119,66 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>G&amp;R Plumbing</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>gandrplumbing.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.gandrplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Drain Installation</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>service@gandrplumbing.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(513) 528-5151</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>100</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>plumbing company Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:13 UTC (cycle 66)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4179,6 +4179,122 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Roby Services</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>robyservicesnow.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://www.robyservicesnow.com/hvac/air-conditioning/installation/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>hello@robyservicesnow.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(704)612-7224</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>AC installation Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Roofing in Ankeny, IA | DLR Construction LLC</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>generalcontractorankenyia.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.generalcontractorankenyia.com/roofing</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>info@dlrconstructionia.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(515) 729-0426</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>86</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>roofing contractor Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:16 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4260,7 +4260,6 @@
           <t>https://www.generalcontractorankenyia.com/roofing</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>info@dlrconstructionia.com</t>
@@ -4290,6 +4289,66 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Wave Roofing</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>waveroofingfayettevillenc.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.waveroofingfayettevillenc.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Licensed Roofer</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>waveroofingfayetteville@gmail.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(910) 613-9300</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>90</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>residential roofing company Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:17 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4354,6 +4354,118 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>HVAC Contactor, Local HVAC Company | Tempe, AZ | Perfection Air</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>perfectionairaz.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://www.perfectionairaz.com/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>allie@perfectionairaz.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(480) 698-3711</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>92</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Thermal Pros HVAC Arizona</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>thermalprosac.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://thermalprosac.com/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>service@thermalpros.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>623-975-0077</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>76</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:19 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4375,7 +4375,6 @@
           <t>https://www.perfectionairaz.com/</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>allie@perfectionairaz.com</t>
@@ -4431,7 +4430,6 @@
           <t>https://thermalprosac.com/</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>service@thermalpros.com</t>
@@ -4461,6 +4459,182 @@
         </is>
       </c>
       <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Integrity Roofing of Florida</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>integrityroofingofflorida.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://integrityroofingofflorida.com/roof-repair-st-petersburg/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Service Areas</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>info@integrityroofingofflorida.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(813) 388-9190</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>100</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>roof repair company St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>PrimeEdge Roofing</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>primeedgeroofingstpetersburg.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://primeedgeroofingstpetersburg.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>More Customer</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>contact@primeedgeroofingstpetersburg.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(727) 966-7472</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>roof repair company St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>B. Griffith Roofing, Inc.</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>bgriffithroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://bgriffithroofingfl.com/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Roofing Replacement</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>bgriffithroofing@aol.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>86</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>roof repair company St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:20 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4615,7 +4615,6 @@
           <t>bgriffithroofing@aol.com</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>St Petersburg FL</t>
@@ -4635,6 +4634,178 @@
         </is>
       </c>
       <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Sewer Line Installation and Repair</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>lambsplumbingva.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.lambsplumbingva.com/sewerlines.html</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>lambsplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(804) 247-0519</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>100</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>sewer repair Richmond VA</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>HVAC Services in Garland, TX | Vortex Air Solutions</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>vortexairsolutions.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.vortexairsolutions.com/garland</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Erik Moreno</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>info@vortexairsolutions.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>469-309-6778</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>HVAC contractor Garland TX</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>USA Pipe Repair</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>usapiperepair.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.usapiperepair.com/services/sewer-repair-richmond-va/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>usapiperepair.office@gmail.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2705140622</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>sewer repair Richmond VA</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:22 UTC (cycle 72)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4660,7 +4660,6 @@
           <t>https://www.lambsplumbingva.com/sewerlines.html</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>lambsplumbing@gmail.com</t>
@@ -4776,7 +4775,6 @@
           <t>https://www.usapiperepair.com/services/sewer-repair-richmond-va/</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>usapiperepair.office@gmail.com</t>
@@ -4806,6 +4804,66 @@
         </is>
       </c>
       <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Air Master Cooling &amp; Heating, LLC</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>airmasterlascruces.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://airmasterlascruces.com/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Las Cruces</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>pbirmingham@airmasterlascruces.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(575) 373-5871</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>86</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>HVAC contractor Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:25 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4869,6 +4869,62 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>One Call Plumbing HVAC</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>onecallhvacsc.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://onecallhvacsc.com/services/air-conditioning/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>onecallsc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(864) 362-8810</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>air conditioning repair Greenville SC</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:28 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4890,7 +4890,6 @@
           <t>https://onecallhvacsc.com/services/air-conditioning/</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>onecallsc@gmail.com</t>
@@ -4920,6 +4919,66 @@
         </is>
       </c>
       <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Beckwith Heating &amp; Cooling, Inc.</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>beckwithheatcool.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://beckwithheatcool.com/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Beckwiths Bruce</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>info@beckwithheatcool.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(330) 923-1333</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>100</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>HVAC contractor Akron OH</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:38 UTC (cycle 83)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4984,6 +4984,66 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Replacement | KMR Electrical &amp; HVAC Services</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>kmrhvac.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://kmrhvac.com/services/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Free Quote</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>kenrob2323@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(855) 691-1472</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Allentown PA</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>90</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>heat pump installation Allentown PA</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:51 UTC (cycle 92)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5044,6 +5044,174 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Renew Plumbing, Rooter, and Leak Detection</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>renewplumbing.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.renewplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>service@renewplumbing.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>541-388-0800</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>90</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>plumber Bend OR</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial Plumbing | Bend, Oregon</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>starkplumbing.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.starkplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>info@starkplumbing.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>541-848-7261</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>90</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>plumber Bend OR</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Bend Plumbing Oregon</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>bendplumbingoregon.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://bendplumbingoregon.com/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>info@bendplumbingoregon.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>76</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>plumber Bend OR</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:53 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5065,7 +5065,6 @@
           <t>https://www.renewplumbing.com/</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>service@renewplumbing.com</t>
@@ -5121,7 +5120,6 @@
           <t>https://www.starkplumbing.com/</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>info@starkplumbing.com</t>
@@ -5187,7 +5185,6 @@
           <t>info@bendplumbingoregon.com</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>Bend OR</t>
@@ -5207,6 +5204,62 @@
         </is>
       </c>
       <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>CIW &amp; Sons Plumbing</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ciwsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://www.ciwsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>estimating@ciwsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>1000056754</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>90</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>plumbing company San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:57 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5230,7 +5230,6 @@
           <t>https://www.ciwsplumbing.com/</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>estimating@ciwsplumbing.com</t>
@@ -5260,6 +5259,66 @@
         </is>
       </c>
       <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Appelhanz Roofing</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>appelhanzroofing.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://appelhanzroofing.com/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>keaton@innovativemediacreators.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(785) 246-0006</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Topeka KS</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>residential roofing company Topeka KS</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 16:59 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5324,6 +5324,122 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Billharz Plumbing &amp; Gas Heating — Queens, NY Since 1927</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>billharzplumbing.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://billharzplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Generation Our</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>info@billharzplumbing.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(718) 784-2468</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>plumbing company Queens NY</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Bryant Iowa Heating and Cooling | Trusted HVAC for Iowa Homes</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>bryantiowahc.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://bryantiowahc.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>info@bryantiowahc.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(515) 963-0333</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>100</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>heating and cooling company Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:02 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5405,7 +5405,6 @@
           <t>https://bryantiowahc.com/</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>info@bryantiowahc.com</t>
@@ -5435,6 +5434,66 @@
         </is>
       </c>
       <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Plumbing Services | Rockford, IL | ProTech Plumbing Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>protechplumbinghvac.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.protechplumbinghvac.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Winnebago County</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>bprotech71@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(815) 621-9382</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>plumbing company Rockford IL</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:03 UTC (cycle 100)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5499,6 +5499,66 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Bravo Mechanical</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>bravomechanicalny.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.bravomechanicalny.com/services/hvac-installation/yonkers</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>What Homeowners</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>info@bravomechanicalny.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(914) 361-9142</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>84</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>AC installation Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:12 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5559,6 +5559,62 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>HVAC Contractor | Fort Lauderdale, Florida</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>americastechnicalservices.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.americastechnicalservices.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>info@atsincfl.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>954-467-6188</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>90</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:14 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5580,7 +5580,6 @@
           <t>https://www.americastechnicalservices.com/</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>info@atsincfl.com</t>
@@ -5610,6 +5609,66 @@
         </is>
       </c>
       <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Craftsman's Plumbing</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>craftsmansplumbing.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://craftsmansplumbing.com/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Emergency Home</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>contact@craftsmansplumbing.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(520) 638-6604</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>90</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>sewer repair Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:22 UTC (cycle 113)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5674,6 +5674,66 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>plumbingprosfortlauderdale.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://plumbingprosfortlauderdale.com/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Point Tamarac</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>service@fortlauderdaleplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(754) 314-3927</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>100</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>plumber Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:25 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5734,6 +5734,66 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>The Drain Smith | Trenchless, Sewer Repair &amp; Hydro Jetting</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>thedrainsmith.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://thedrainsmith.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Rated Sewer</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>info@thedrainsmith.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>513-402-0242</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>84</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>sewer repair Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:31 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5794,6 +5794,62 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Morrissey Construction LLC</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>morrisseyconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.morrisseyconstructionllc.com/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>matthew@morrisseyconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>860-657-9346</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Hartford CT</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>100</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>roof repair company Hartford CT</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:33 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5815,7 +5815,6 @@
           <t>https://www.morrisseyconstructionllc.com/</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>matthew@morrisseyconstructionllc.com</t>
@@ -5845,6 +5844,66 @@
         </is>
       </c>
       <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Bounds Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>boundshvac.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://boundshvac.com/air-conditioning/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Bounds Heating</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>analytics@graystats.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>352-472-2761</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>100</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>air conditioning repair Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:40 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5909,6 +5909,122 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>A STAR Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>astarairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.astarairconditioning.com/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>astarfl@gmail.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(800) 454-0987</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>100</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>heating and cooling company Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Creative Metal Systems LLC</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>creativemetalsystems.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://creativemetalsystems.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>East Tennessee</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>brian@creativemetalsystems.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>865.738.8962</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Knoxville TN</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>80</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Knoxville TN</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:42 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5930,7 +5930,6 @@
           <t>https://www.astarairconditioning.com/</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>astarfl@gmail.com</t>
@@ -6020,6 +6019,122 @@
         </is>
       </c>
       <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Laurel Home Improvements</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>lhiwenailit.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://lhiwenailit.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Jeff Carter</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>info@lhiwenailit.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>304-296-2050</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Morgantown WV</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>96</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>roof repair company Morgantown WV</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Mason Air Systems</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>masonairsystems.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://masonairsystems.com/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>info@masonairsystems.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(361) 808-9161</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>heating and cooling company Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:43 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6105,7 +6105,6 @@
           <t>https://masonairsystems.com/</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>info@masonairsystems.com</t>
@@ -6135,6 +6134,58 @@
         </is>
       </c>
       <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Lh Heating</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>lhheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.lhheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>lemonte@lhheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>62</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>HVAC contractor Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:45 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6160,13 +6160,11 @@
           <t>https://www.lhheatingandair.com/</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>lemonte@lhheatingandair.com</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>Chattanooga TN</t>
@@ -6186,6 +6184,178 @@
         </is>
       </c>
       <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Plumber | Plumber Myrtle Beach | Plumber Near Me | Emergency Plumbing - Emergenc</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>plumber-myrtlebeach.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://plumber-myrtlebeach.com/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>eplumbing247@gmail.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>843-286 3158</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>100</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>emergency plumber Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Horn Brothers Roofing | Expert Residential &amp; Commercial Roofing in Colorado</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>hornbrothersroofing.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://hornbrothersroofing.com/local/metal-roofing/westminster/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Roofing Horn</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>info@hornbrothersroofing.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(303) 274-1111</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>96</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Westminster CO</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>USA PLUMBING</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>usaplumbingsc.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.usaplumbingsc.com/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>usaplumbing@outlook.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>843-241-8054</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>88</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>emergency plumber Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:46 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6210,7 +6210,6 @@
           <t>https://plumber-myrtlebeach.com/</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>eplumbing247@gmail.com</t>
@@ -6326,7 +6325,6 @@
           <t>https://www.usaplumbingsc.com/</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>usaplumbing@outlook.com</t>
@@ -6356,6 +6354,126 @@
         </is>
       </c>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Roof Installation &amp; Replacement | Richmond, VA</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>jacobsladder.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.jacobsladder.com/roof-installation-and-replacement</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Why Richmond</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>sales@jacobsladder.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(804) 597-0215</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>roof replacement Richmond VA</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Philadelphia Roofer | Philly's Phinest Roofing</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>phillysphinestroofing.net</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://phillysphinestroofing.net/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Blogs Contact</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>phillysphinestroofers@gmail.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(267) 343-8469</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>98</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>roofer Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:48 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6479,6 +6479,66 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Story Roofing</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>storyroofing.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://storyroofing.com/metal-roof-installation-cape-coral/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>info@storyroofing.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(231) 269-3210</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>74</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 17:49 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6539,6 +6539,62 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>One Way Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>onewayair.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.onewayair.com/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>onewayair@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>(310) 212-5554</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>100</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>heating and cooling company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:03 UTC (cycle 140)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6560,7 +6560,6 @@
           <t>https://www.onewayair.com/</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>onewayair@hotmail.com</t>
@@ -6590,6 +6589,62 @@
         </is>
       </c>
       <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Air Conditioning Installation, AC Replacement: Concord, NC | Heat &amp; Air Direct b</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>heatandairdirect.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.heatandairdirect.com/ac-installations</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>russ@heatandairdirect.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(704) 918-5421</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>86</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>AC installation Concord NC</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:06 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6615,7 +6615,6 @@
           <t>https://www.heatandairdirect.com/ac-installations</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>russ@heatandairdirect.com</t>
@@ -6645,6 +6644,66 @@
         </is>
       </c>
       <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Heat Pumps</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>hometownairnc.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://hometownairnc.com/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Triangle Region</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@hometownairnc.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>919-568-3212</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>heat pump installation Durham NC</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:19 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6709,6 +6709,66 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>North Star Contracting</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>northstarroofingak.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.northstarroofingak.com/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Eagle River</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>alaska@north-star.us</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(907) 903-7068</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>100</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>roof replacement Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:25 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6769,6 +6769,62 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Waggoner Roofing &amp; Restorations (Copy)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>waggonerroofing.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.waggonerroofing.com/pasadena-tx</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Waggoner Roofing</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>tyler@waggonerroofing.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>76</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>residential roofing company Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:26 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6800,7 +6800,6 @@
           <t>tyler@waggonerroofing.com</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
           <t>Pasadena TX</t>
@@ -6820,6 +6819,66 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>HVAC Installation &amp; Repair | DNA Heating and Cooling | los angeles, CA</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>dnaheatingandcooling.org</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.dnaheatingandcooling.org/santa-clarita--ca</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>dnahvacr@gmail.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>818-806-7750</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>96</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>heating and cooling company Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:31 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6884,6 +6884,122 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation and Replacement in Ankeny, IA</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>ankeny-ia.centralheatairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://ankeny-ia.centralheatairconditioning.com/heat-pump-installation-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>contact@centralheatairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>(833) 435-6630</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>heat pump installation Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Ankeny, IA | Year-Round</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ankeny-ia.flphvacservices.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://ankeny-ia.flphvacservices.com/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Indoor Air</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>contact@flphvacservices.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(833) 963-1661</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>90</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>heat pump installation Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:32 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6905,7 +6905,6 @@
           <t>https://ankeny-ia.centralheatairconditioning.com/heat-pump-installation-and-replacement/</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>contact@centralheatairconditioning.com</t>
@@ -6995,6 +6994,126 @@
         </is>
       </c>
       <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Comfort Pro Home Services</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>comfortprohome.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://comfortprohome.com/fresno/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Comfort Pro</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>info@comfortprohome.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>559-354-0035</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>100</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>heating and cooling company Fresno CA</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>A&amp;A Plumbing - Omaha Plumbers - Commercial Plumbing - residential plumbing - oma</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>anaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://anaplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Projects Specials</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>anaplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(402) 932-3899</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>88</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>plumber Omaha NE</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:35 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7119,6 +7119,66 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>greater front range roofing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>gfrroofing.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://gfrroofing.com/roofing-thornton-co/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>matt@gfrroofing.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>970-988-2341</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>roofing contractor Thornton CO</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:44 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7179,6 +7179,126 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>First Chicago Plumbing</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>firstchicagoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://firstchicagoplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Eugene Petrov</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>info@firstchicagoplumbing.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>(847) 262-4244</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>90</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>plumber Chicago IL</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Chicago Drain Masters Plumbing 24/7 | Expert Plumber in Chicago, IL</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>chicagodrainmasters.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://chicagodrainmasters.com/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Why Chicago</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>info@chicagodrainmasters.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(464) 245-3033</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>90</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>plumber Chicago IL</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:51 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7299,6 +7299,66 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>TCR</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>tri-cities-roofing.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.tri-cities-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>contact@tri-cities-roofing.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>423.268.4240</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>roofer Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 18:54 UTC (cycle 175)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7359,6 +7359,126 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Ham Plumbing</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>hamplumbing.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.hamplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Layton Ha</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>931-572-7220</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>92</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>plumber Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Emergency Plumbing in Clarksville, Tennessee | Fast Local Response</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>clarksvilleplumbers.us</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://clarksvilleplumbers.us/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Michael Reynolds</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>service@clarksvilleplumbers.us</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(931) 208-8763</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>plumber Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 19:00 UTC (cycle 179)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7479,6 +7479,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Roof Inspection &amp; Repair - Escondido, CA - Alfredo’s Roofing</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>alfredos-roofing.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://www.alfredos-roofing.com/roof-installation-repair-replacement</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>alfredoroofing64@gmail.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(760) 473-2667</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>90</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>roof repair company Escondido CA</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 19:05 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7539,6 +7539,66 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Lincoln Nebraska</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>coalitionrestoration.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://coalitionrestoration.com/nebraska/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Ashley Ndukwu</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>sheena@crestorationc.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(469) 609-1994</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>80</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>roofing contractor Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 19:12 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7599,6 +7599,66 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Peake Roofing</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>peakeroofingoh.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://peakeroofingoh.com/cincinnati-oh/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Yours At</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>sales@peakeroofingoh.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>513-832-0024</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>98</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>roof repair company Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 19:20 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7659,6 +7659,66 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Reliance Air Services</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>relianceairservices.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://relianceairservices.com/heat-pump-installation-sarasota-fl</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>xavier@relianceairservices.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(941) 417-4848</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>90</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>heat pump installation Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 19:30 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7719,6 +7719,62 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Michigan Drain &amp;amp; Sewer</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>misewer.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://misewer.com/</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>michigansewer@gmail.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(810) 519-2005</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Flint MI</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>88</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>sewer repair Flint MI</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 19:31 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7740,7 +7740,6 @@
           <t>https://misewer.com/</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>michigansewer@gmail.com</t>
@@ -7770,6 +7769,62 @@
         </is>
       </c>
       <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Ohio City Heating And Cooling LLC</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>ohiocityhvac.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://www.ohiocityhvac.com/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Comfort You</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>ohiocityhvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Cleveland OH</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>76</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>heating and cooling company Cleveland OH</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:42 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7805,7 +7805,6 @@
           <t>ohiocityhvac@gmail.com</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>Cleveland OH</t>
@@ -7825,6 +7824,66 @@
         </is>
       </c>
       <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Plano No-Dig Pipe Repair</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>planopiperepair.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://planopiperepair.com/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Request Free</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>dispatch@planonodigpipe.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>(877) 552-8556</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>84</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>sewer repair Plano TX</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:43 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7889,6 +7889,122 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Comfy Castle Heating and Air</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>comfycastlehvac.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://www.comfycastlehvac.com/air-conditioner/installation-lakewood</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Expert Nathan</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>comfycastlehvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(303) 227-9999</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>84</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>AC installation Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Greensboro Water Heater Service: Replace Water Heater</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>edwardsandmillsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://edwardsandmillsplumbing.com/services-water-heaters.php</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>edmills@bellsouth.net</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(336) 299-6309</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Greensboro NC</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>74</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>water heater repair Greensboro NC</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:46 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7970,7 +7970,6 @@
           <t>https://edwardsandmillsplumbing.com/services-water-heaters.php</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>edmills@bellsouth.net</t>
@@ -8000,6 +7999,62 @@
         </is>
       </c>
       <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Evolution Air HVAC</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>evolutionairllc.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://evolutionairllc.com/</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>service@evolutionairllc.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(203) 724-9814</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>90</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>air conditioning repair Stamford CT</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:48 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8025,7 +8025,6 @@
           <t>https://evolutionairllc.com/</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>service@evolutionairllc.com</t>
@@ -8055,6 +8054,122 @@
         </is>
       </c>
       <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Roofing Ocala</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>roofingandrepairocala.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://roofingandrepairocala.com/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Emergency Roofing</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>info@info.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(352) 425-4421</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>90</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>roof repair company Ocala FL</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Home | Texas Air &amp; Heat</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>txairheat.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.txairheat.com/</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Grand Prairie</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>info@txairheat.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>76</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>HVAC contractor Arlington TX</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:51 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8150,7 +8150,6 @@
           <t>info@txairheat.com</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>Arlington TX</t>
@@ -8170,6 +8169,66 @@
         </is>
       </c>
       <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Roofing in Bethlehem, PA | Roof Replacement &amp; Repair | LV Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>lvroofingpa.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://lvroofingpa.com/roofing-bethlehem-pa/</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Lehigh Valley</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>estimates@lvroofingpa.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(835) 248-0004</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>100</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>roof replacement Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:52 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8234,6 +8234,66 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Residential Roofing - Fresno, CA - Allstate Roofing Inc.</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>allstateroofingcompany.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.allstateroofingcompany.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Shingles Certainteed</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>allstateroofingincfresno@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>559-325-2286</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>84</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>residential roofing company Fresno CA</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:54 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8294,6 +8294,62 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>HVAC Services | Corpus Christi, TX | LTJ Air</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ltjair.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.ltjair.com/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>ltjr2005@gmail.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(361) 249-4039</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>96</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>air conditioning repair Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:55 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8315,7 +8315,6 @@
           <t>https://www.ltjair.com/</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>ltjr2005@gmail.com</t>
@@ -8345,6 +8344,66 @@
         </is>
       </c>
       <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Bacon Roofing</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>baconroofing.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://baconroofing.com/service-area/mesquite-roofing-contractor/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Decades Bacon</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>info@baconroofing.com</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>972-772-1999</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Mesquite TX</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>100</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>roofing contractor Mesquite TX</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 20:59 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8409,6 +8409,62 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>California Bay Roofing Inc</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>calbayroofing.net</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://www.californiabayroofinginc.net/fremont-roofing</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>calbayroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>(415) 684-4498</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>100</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>roofer Fremont CA</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:07 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L138"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8430,7 +8430,6 @@
           <t>https://www.californiabayroofinginc.net/fremont-roofing</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>calbayroofinginc@gmail.com</t>
@@ -8460,6 +8459,66 @@
         </is>
       </c>
       <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>OnPoint Roofing</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>onpointroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://onpointroofingfl.com/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Central Florida</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>brandon@onpointroofingfl.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>321 666 5819</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>100</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Orlando FL</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:08 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8524,6 +8524,122 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Visocchi Roofing Company</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>visocchiroofing.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://visocchiroofing.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Chris Visocchi</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>cvisocchi@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>(781) 953-1508</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>90</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Boston MA</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Roofing Services in Brockton, MA</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>froof.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://www.froof.com/brockton-ma</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Company In</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>support@froof.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Brockton MA</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>62</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>roofer Brockton MA</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:17 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8615,7 +8615,6 @@
           <t>support@froof.com</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
           <t>Brockton MA</t>
@@ -8635,6 +8634,186 @@
         </is>
       </c>
       <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Cary, NC - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>caryhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://caryhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Cary Towne</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>info@caryhvacpros.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>(919) 752-3826</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Cary NC</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>100</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>heating and cooling company Cary NC</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Aaron's Custom Plumbing Services | Santa Fe, NM Plumbers</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>aaronscustomplumbing.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://aaronscustomplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Helen Wulfers</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>aaronscustomplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>1505806131</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>100</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>plumbing company Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Gabriel's Plumbing &amp; HVAC</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>gabrielsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://gabrielsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Northern New</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>gabrielsplumbingandhvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(505) 469-8517</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>98</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>plumbing company Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:19 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8819,6 +8819,66 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Bodensteiner Service Inc.</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>bsiairhouston.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://www.bsiairhouston.com/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Service Technician</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>bsiairhtx@gmail.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>713-868-0050</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>100</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>furnace repair Houston TX</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:20 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8879,6 +8879,66 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>covenantplumbing.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://covenantplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Middle Georgia</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>service@covenantplumbing.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>478-745-7436</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Macon GA</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>76</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>plumbing company Macon GA</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:25 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8939,6 +8939,62 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>roofwithrouse.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://roofwithrouse.com/</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>coveryourhouse@gmail.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(916) 707-1682</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>90</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>roofer Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:33 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L147"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8960,7 +8960,6 @@
           <t>https://roofwithrouse.com/</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
           <t>coveryourhouse@gmail.com</t>
@@ -8990,6 +8989,62 @@
         </is>
       </c>
       <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Jasmor Properties LLC</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>jasmorprop.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://jasmorprop.com/services/roof-repair/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>jasmorprop@gmail.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>(603) 961-0335</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Concord NH</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>100</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>roof repair company Concord NH</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:38 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9015,7 +9015,6 @@
           <t>https://jasmorprop.com/services/roof-repair/</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>jasmorprop@gmail.com</t>
@@ -9045,6 +9044,62 @@
         </is>
       </c>
       <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Water Heater Repair in Rockford, IL | Fast Service</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>plumberrockfordil.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://www.plumberrockfordil.com/services/water-heater-repair.html</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>info@plumberrockfordil.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(815) 399 5617</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>90</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>water heater repair Rockford IL</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:39 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L149"/>
+  <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9070,7 +9070,6 @@
           <t>https://www.plumberrockfordil.com/services/water-heater-repair.html</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
           <t>info@plumberrockfordil.com</t>
@@ -9100,6 +9099,242 @@
         </is>
       </c>
       <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Mr. Plumber Inc</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>mrplumber.nyc</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://mrplumber.nyc/</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>mrplumbernyc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>347-565-5130</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>100</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>plumber Bronx NY</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>New York Plumbing Directory</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>newyorkplumbingdirectory.com</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://www.newyorkplumbingdirectory.com/plumbers/new-york/the-bronx</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>contact@newyorkplumbingdirectory.com</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>(914) 291-3274</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>100</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>plumber Bronx NY</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Mathis Home Improvements, Inc.</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>mathishomeimprovements.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://www.mathishomeimprovements.com/metal-roofs</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Better Business</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>office@mathishomeimprovements.com</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>336-744-1141</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>90</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>HVAC Experts| Cool Kings Heating and Air | Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>coolkingsheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://www.coolkingsheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Air Our</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>office@coolkingshvac.com</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>(225) 681-2665</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>86</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>HVAC contractor Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:42 UTC (cycle 44)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9125,7 +9125,6 @@
           <t>https://mrplumber.nyc/</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>mrplumbernyc@gmail.com</t>
@@ -9335,6 +9334,62 @@
         </is>
       </c>
       <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Plumbing Company |Tyler' Plumbing Heating &amp; Cooling | South Bend, IN</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>tylersheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://www.tylersheatingandcooling.com/plumbing-company-south-bend-in</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>casey@tylersphc.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>(574) 347-4225</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>South Bend IN</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>100</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>plumbing company South Bend IN</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:55 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9360,7 +9360,6 @@
           <t>https://www.tylersheatingandcooling.com/plumbing-company-south-bend-in</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>casey@tylersphc.com</t>
@@ -9390,6 +9389,122 @@
         </is>
       </c>
       <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>HVAC &amp; Refrigeration Services | Burlington VT and Surrounding Areas | Kirk Mecha</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>kirkmechanical.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://www.kirkmechanical.com/</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>bill@kirkmechanical.com</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>(802) 999-7452</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>90</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>AC installation Burlington VT</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Central Air Installation Burlington, VT</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>hvac4pro.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://hvac4pro.com/central-air-installation-burlington-vt/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Burlington Homeowner</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>info@hvac4pro.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>(833) 435-3815</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>90</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>AC installation Burlington VT</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 21:58 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9415,7 +9415,6 @@
           <t>https://www.kirkmechanical.com/</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>bill@kirkmechanical.com</t>
@@ -9505,6 +9504,62 @@
         </is>
       </c>
       <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Kool Mode AC and Heating</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>koolmodehvac.com</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://koolmodehvac.com/</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>nkoolmode@gmail.com</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>(281) 212-7629</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>88</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>heating and cooling company Katy TX</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:07 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L157"/>
+  <dimension ref="A1:L158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9530,7 +9530,6 @@
           <t>https://koolmodehvac.com/</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
       <c r="F157" t="inlineStr">
         <is>
           <t>nkoolmode@gmail.com</t>
@@ -9560,6 +9559,62 @@
         </is>
       </c>
       <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Aqua Inc.</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>aquainc.com</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://aquainc.com/our-services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>info@aquainc.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>407-584-1001</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>90</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>sewer repair Orlando FL</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:10 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L158"/>
+  <dimension ref="A1:L159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9585,7 +9585,6 @@
           <t>https://aquainc.com/our-services/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr">
         <is>
           <t>info@aquainc.com</t>
@@ -9615,6 +9614,66 @@
         </is>
       </c>
       <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Integrity Roofing and Repair</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>integrityroofingandrepair.com</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://integrityroofingandrepair.com/</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Integrity Roofing</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>integrityroofingandrepairllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>(509) 655-0090</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>98</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>roof repair company Spokane WA</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:29 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L159"/>
+  <dimension ref="A1:L161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9679,6 +9679,126 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Jones Plumbing</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>jonesplumbingtx.com</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://www.jonesplumbingtx.com/</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Responsible Master</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>jonesplumbing2022@gmail.com</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>830-708-3795</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>90</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>plumber New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Plumber Services | New Braunfels, TX | Blackburn Plumbing</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>blackburnplumbingtx.com</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://www.blackburnplumbingtx.com/</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Homeowners Can</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>service@blackburnplumbingtx.com</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>(210) 630-2593</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>90</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>plumber New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:30 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L161"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9799,6 +9799,114 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Aire-Craft Heating &amp; Cooling Co Inc | Heating Baltimore</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>airecrafthvac.com</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://www.airecrafthvac.com/</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>airecraftoffice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>74</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>heating and cooling company Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>coldspringhvac.com</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>http://www.coldspringhvac.com/</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>info@companyname.com</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>(410) 367-8719</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>64</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>heating and cooling company Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:41 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9820,13 +9820,11 @@
           <t>https://www.airecrafthvac.com/</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
           <t>airecraftoffice@gmail.com</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
           <t>Baltimore MD</t>
@@ -9872,7 +9870,6 @@
           <t>http://www.coldspringhvac.com/</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
           <t>info@companyname.com</t>
@@ -9902,6 +9899,66 @@
         </is>
       </c>
       <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Nevados A/C Services LLC</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>nevadosacservices.com</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://nevadosacservices.com/</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>acnevados@gmail.com</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>(786) 366 1317</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>86</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>AC installation Miramar FL</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:42 UTC (cycle 85)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9964,6 +9964,66 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Watts Roofing Home</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>residentialroofingcolumbia.com</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://www.residentialroofingcolumbia.com/</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>john@doe.com</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>803-786-4610</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>96</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>residential roofing company Columbia SC</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:44 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L165"/>
+  <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10024,6 +10024,62 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Heat Pump Repair and Mini Split Installation in Sugar Land, TX</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>multipointacheat.com</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://multipointacheat.com/service-areas/sugar-land-tx</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>info@multipointacheat.com</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>8329633789</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>90</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>heat pump installation Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:51 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L166"/>
+  <dimension ref="A1:L167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10045,7 +10045,6 @@
           <t>https://multipointacheat.com/service-areas/sugar-land-tx</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>info@multipointacheat.com</t>
@@ -10075,6 +10074,62 @@
         </is>
       </c>
       <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>5150 Heating and Air Conditioning, LLC</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>business.casperwyoming.org</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://business.casperwyoming.org/list/member/5150-heating-and-air-conditioning-llc-17569</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>information@casperwyoming.org</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>(307) 259-0053</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Casper WY</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>98</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>air conditioning repair Casper WY</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:54 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L167"/>
+  <dimension ref="A1:L168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10100,7 +10100,6 @@
           <t>https://business.casperwyoming.org/list/member/5150-heating-and-air-conditioning-llc-17569</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
           <t>information@casperwyoming.org</t>
@@ -10130,6 +10129,66 @@
         </is>
       </c>
       <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Straight Shooter</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>straightshooter.ac</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://straightshooter.ac/</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>support@straightshooter.ac</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>858-935-4328</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>100</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>heating and cooling company San Diego CA</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:56 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L168"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10194,6 +10194,122 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Manasota Cooling &amp; Heating LLC</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>manasotacooling.com</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://manasotacooling.com/</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Southwest Florid</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>alex@manasotacooling.com</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>941-352-0977</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>100</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>heating and cooling company Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Heating and Air Conditioner Repair Sarasota FL | HVAC Sarasota FL</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>montgomeryair.com</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://www.montgomeryair.com/sarasota-fl</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Manatee County</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>support@gethearth.com</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>74</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>heating and cooling company Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 22:58 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L170"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10285,7 +10285,6 @@
           <t>support@gethearth.com</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr">
         <is>
           <t>Sarasota FL</t>
@@ -10305,6 +10304,66 @@
         </is>
       </c>
       <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Trusted Raleigh Roofing Company</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>arcroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://arcroofingconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Raleigh Roofing</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>info@arcroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>984-237-2775</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>86</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>roofing contractor Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:00 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:L172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10369,6 +10369,66 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Old Fashioned Roofing</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>oldfashionedroofing.com</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://www.oldfashionedroofing.com/service-areas/kenosha-wi/</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Old Fashioned</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>admin@oldfashionedroofing.com</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>262-229-8909</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Kenosha WI</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>98</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>roofer Kenosha WI</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:13 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L172"/>
+  <dimension ref="A1:L173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10429,6 +10429,66 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Pair of Aces A/C LLC</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>pairofacesacllc.com</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://pairofacesacllc.com/</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Greater Houston</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>pairofacesac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>832-519-7178</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>100</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>furnace repair McAllen TX</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:16 UTC (cycle 108)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L173"/>
+  <dimension ref="A1:L175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10489,6 +10489,126 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>All One Exteriors</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>alloneexteriors.com</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://alloneexteriors.com/service-areas/gary-in</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Reviews Family</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>info@alloneexteriors.com</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>(219) 400-0223</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>100</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>roof replacement Gary IN</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Imagine Roofs</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>imagineroofs.com</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://www.imagineroofs.com/gary-roofing</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Miller Beach</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>joshua@imagineroofs.com</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>219-250-1908</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>86</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>roof replacement Gary IN</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:19 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10609,6 +10609,66 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>HVAC Services Coral| Rapid Cool LLC | Coral Springs, FL</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>rapidcoolac.com</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://www.rapidcoolac.com/coral-springs-fl</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Expert Solutions</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>rapidcoolacrepair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>(754) 610-4831</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>90</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>heating and cooling company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:26 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L176"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10669,6 +10669,62 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>24/7 Emergency Plumbing in Meridian, ID | Meridian Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>meridianplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://www.meridianplumbingservices.com/services/emergency-plumbing/</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>info@meridianplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>(205) 627-7185</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Meridian ID</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>90</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>emergency plumber Meridian ID</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:28 UTC (cycle 116)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10690,7 +10690,6 @@
           <t>https://www.meridianplumbingservices.com/services/emergency-plumbing/</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
           <t>info@meridianplumbingservices.com</t>
@@ -10720,6 +10719,118 @@
         </is>
       </c>
       <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Frontier Plumbing</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>frontier-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://frontier-plumbing.com/</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>info@frontier-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>(661) 589-6203</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>100</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>plumber Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Stone Plumbing and Heating</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>stoneplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://stoneplumbingheating.com/</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>office@stoneplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>218-525-4450</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>80</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>plumbing company Duluth MN</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:38 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10745,7 +10745,6 @@
           <t>https://frontier-plumbing.com/</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
           <t>info@frontier-plumbing.com</t>
@@ -10801,7 +10800,6 @@
           <t>https://stoneplumbingheating.com/</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
           <t>office@stoneplumbingheating.com</t>
@@ -10831,6 +10829,126 @@
         </is>
       </c>
       <c r="L179" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Davis Roofing Co Inc</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>davisroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://davisroofinginc.com/service-areas/winston-salem/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Davis Ro</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>sam@davisroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>336-431-6485</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>100</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Providence Roofing</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>providenceroofs.com</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://providenceroofs.com/service-areas/winston-salem/</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>At Providence</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>info@providenceroofs.com</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>704-883-6052</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>90</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:45 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10954,6 +10954,62 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>1UP Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>1upheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://1upheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>mainuser@1upheating.com</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>(412) 452-6806</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>90</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>heating and cooling company Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:47 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L182"/>
+  <dimension ref="A1:L183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10975,7 +10975,6 @@
           <t>https://1upheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
           <t>mainuser@1upheating.com</t>
@@ -11005,6 +11004,66 @@
         </is>
       </c>
       <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Day Night HVAC &amp; Plumbing Inc.</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>daynighthvacplumbing.com</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://daynighthvacplumbing.com/ac-services/air-conditioning-repair-queens/</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Serving Forest</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>info@daynighthvacplumbing.com</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>718-518-2041</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>90</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>air conditioning repair Queens NY</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-02 23:51 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-02.xlsx
+++ b/output/leads_2026-10-02.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L183"/>
+  <dimension ref="A1:L184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11069,6 +11069,62 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Emergency Plumbing | Cape Coral &amp; Marco Island, FL</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>monahansplumbing.com</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://www.monahansplumbing.com/emergency-services-plumbing-repair</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>monahanspipes@aol.com</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>(239) 541-9527</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>90</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>emergency plumber Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>